<commit_message>
Recalibrate Virgen del Valle production to 113 units (cap 120)
Previous model overstated need by projecting full Sept+Oct horizon
while under-counting existing VELA+TALLER pool (~32 days coverage).

New logic: post-peak coverage by size (20d VELA floor + 14d WEB
incremental), TALLER only 15% as immediate store replenishment.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SPOTS_VIRGEN_PRODUCCION_SUGERIDA.xlsx
+++ b/SPOTS_VIRGEN_PRODUCCION_SUGERIDA.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sept + mitad octubre</t>
+          <t>Cobertura 20d VELA + WEB (base)</t>
         </is>
       </c>
     </row>
@@ -581,102 +581,122 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Demanda proyectada VELA</t>
+          <t>Cobertura pool actual (días @ post-pico)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>303</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Demanda proyectada WEB (35%)</t>
+          <t>Objetivo cobertura VELA (días)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>107</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Producción sugerida total</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>295</v>
+          <t>Incremento WEB (33%)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>14 días</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Producción bruta (sin tope)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Supuestos</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
+          <t>Producción sugerida total</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>WEB vs VELA</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>30–40% (base 35%)</t>
-        </is>
+          <t>Tope recomendado</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Stock seguridad</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>+12%</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TALLER en cobertura</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>55% del stock</t>
-        </is>
-      </c>
+          <t>Supuestos</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Octubre (mitad)</t>
+          <t>Metodología</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>×0.88 vs ritmo sept</t>
+          <t>Quiebres por talla + WEB · no duplica horizonte calendario completo</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pico</t>
+          <t>Pool VELA+TALLER</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Primeros 4 días ≈ 77% ventas sept</t>
+          <t>110+157 und (~31.9 días post-pico)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TALLER en plan tienda</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>15% puede reponer VELA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>WEB vs VELA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>30–40% (base 33%)</t>
         </is>
       </c>
     </row>
@@ -691,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -746,13 +766,13 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
         <v>19</v>
@@ -770,13 +790,13 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="E3" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
         <v>15</v>
@@ -794,13 +814,13 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="D4" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E4" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
         <v>12</v>
@@ -809,49 +829,49 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>XS</t>
+          <t>XL</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DAMA</t>
+          <t>CAB</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>2XL</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
         <v>13</v>
-      </c>
-      <c r="F6" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -862,20 +882,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>XS</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="D7" t="n">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="E7" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -886,35 +906,83 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D8" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="D9" t="n">
+        <v>37</v>
+      </c>
+      <c r="E9" t="n">
+        <v>9</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" s="2" t="n">
-        <v>295</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1035,19 +1103,19 @@
         <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L3" s="6" t="n">
         <v>30.6</v>
@@ -1075,19 +1143,19 @@
         <v>0</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="L4" s="6" t="n">
         <v>12.7</v>
@@ -1115,19 +1183,19 @@
         <v>0</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>9.1</v>
@@ -1155,19 +1223,19 @@
         <v>0</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>0</v>
+        <v>36</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L6" s="6" t="n">
         <v>90.7</v>
@@ -1195,19 +1263,19 @@
         <v>0</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>0</v>
+        <v>28</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>89.2</v>
@@ -1233,19 +1301,19 @@
         <v>0</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>127</v>
+        <v>70</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>171</v>
+        <v>87</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>126</v>
+        <v>165</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="L8" s="8" t="n"/>
     </row>
@@ -1371,19 +1439,19 @@
         <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="L3" s="6" t="n">
         <v>4.9</v>
@@ -1411,19 +1479,19 @@
         <v>0</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="L4" s="6" t="n">
         <v>9.800000000000001</v>
@@ -1451,19 +1519,19 @@
         <v>0</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>91</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="K5" s="7" t="n">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>2.1</v>
@@ -1491,19 +1559,19 @@
         <v>0</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="L6" s="6" t="n">
         <v>13.5</v>
@@ -1529,19 +1597,19 @@
         <v>0</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>176</v>
+        <v>97</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>237</v>
+        <v>119</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="L7" s="8" t="n"/>
     </row>
@@ -1602,101 +1670,101 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Resto septiembre</t>
+          <t>Cobertura 18d VELA + WEB</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D2" t="n">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="E2" t="n">
-        <v>192</v>
+        <v>150</v>
       </c>
       <c r="F2" t="n">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="G2" t="n">
-        <v>260</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sept + mitad octubre</t>
+          <t>Cobertura 20d VELA + WEB (base)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" t="n">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="E3" t="n">
-        <v>303</v>
+        <v>167</v>
       </c>
       <c r="F3" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="G3" t="n">
-        <v>409</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sept + mitad oct (WEB 30%)</t>
+          <t>Cobertura 20d · WEB 30%</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
         <v>0.3</v>
       </c>
       <c r="E4" t="n">
-        <v>303</v>
+        <v>167</v>
       </c>
       <c r="F4" t="n">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="G4" t="n">
-        <v>393</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sept + mitad oct (WEB 40%)</t>
+          <t>Resto sept post-pico (referencia)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>303</v>
+        <v>184</v>
       </c>
       <c r="F5" t="n">
-        <v>121</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>424</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Document gender/talla curve alignment (DAMA predominance)
Use September sales curve for mix (gen share × talla within gen).
Add dashboard comparison of ventas vs production curves.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SPOTS_VIRGEN_PRODUCCION_SUGERIDA.xlsx
+++ b/SPOTS_VIRGEN_PRODUCCION_SUGERIDA.xlsx
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15">
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16">
@@ -790,13 +790,13 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
         <v>24</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
         <v>15</v>
@@ -817,7 +817,7 @@
         <v>18</v>
       </c>
       <c r="D4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E4" t="n">
         <v>6</v>
@@ -886,10 +886,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7" t="n">
         <v>6</v>
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D8" t="n">
         <v>20</v>
@@ -937,7 +937,7 @@
         <v>39</v>
       </c>
       <c r="D9" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E9" t="n">
         <v>9</v>
@@ -978,7 +978,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" s="2" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>8</v>
@@ -1118,7 +1118,7 @@
         <v>3</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>30.6</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="4">
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>14.1</v>
+        <v>14.4</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>16</v>
@@ -1146,19 +1146,19 @@
         <v>24</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>35</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="5">
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>18</v>
@@ -1183,7 +1183,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>6</v>
@@ -1198,7 +1198,7 @@
         <v>18</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>9.1</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>3</v>
@@ -1238,7 +1238,7 @@
         <v>1</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>90.7</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>2</v>
@@ -1278,7 +1278,7 @@
         <v>1</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>89.2</v>
+        <v>86.3</v>
       </c>
     </row>
     <row r="8">
@@ -1301,19 +1301,19 @@
         <v>0</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>165</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L8" s="8" t="n"/>
     </row>
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>14.7</v>
+        <v>14.4</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>16</v>
@@ -1439,7 +1439,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H3" s="6" t="n">
         <v>6</v>
@@ -1451,10 +1451,10 @@
         <v>23</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>12.3</v>
+        <v>11.7</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>13</v>
@@ -1485,16 +1485,16 @@
         <v>5</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>30</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="5">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>22.3</v>
+        <v>22.5</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>25</v>
@@ -1519,7 +1519,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>9</v>
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>10</v>
@@ -1565,7 +1565,7 @@
         <v>3</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>25</v>
@@ -1574,7 +1574,7 @@
         <v>6</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>13.5</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="7">
@@ -1609,7 +1609,7 @@
         <v>102</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L7" s="8" t="n"/>
     </row>

</xml_diff>

<commit_message>
Format Virgen production Excel like SPOTS expansion matrix
Add PRODUCCION sheet with CAB/DAMA blocks, tallas as columns,
design/color rows, TOTAL per gender, and ventas sept reference curve.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SPOTS_VIRGEN_PRODUCCION_SUGERIDA.xlsx
+++ b/SPOTS_VIRGEN_PRODUCCION_SUGERIDA.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PEDIDO_TS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PRODUCCION" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="CAB" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="DAMA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ESCENARIOS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="PEDIDO_TS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ESCENARIOS" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,14 +40,32 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -95,13 +119,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -110,12 +134,20 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -711,6 +743,616 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>SPOTS Virgen del Valle — Producción sugerida · Margarita (VELA) + WEB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>CAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>CANTIDADES POR DISEÑO / COLOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SPOTS MANGA CORTA CAB — Virgen del Valle · VELA + WEB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>2XL</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Virgen del Valle (Blanco)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>↳ Ref. ventas sept (curva)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>CANTIDADES POR DISEÑO / COLOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SPOTS MANGA CORTA DAMA — Virgen del Valle · VELA + WEB</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Virgen del Valle (Blanco)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="7" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>↳ Ref. ventas sept (curva)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="8" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="10" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL PRODUCCIÓN SUGERIDA</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>SPOTS MANGA CORTA — Virgen del Valle · VELA + WEB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>CANTIDADES POR DISEÑO / COLOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SPOTS MANGA CORTA CAB — Virgen del Valle · VELA + WEB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>2XL</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Virgen del Valle (Blanco)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>↳ Ref. ventas sept (curva)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL CAB</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>SPOTS MANGA CORTA — Virgen del Valle · VELA + WEB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>CANTIDADES POR DISEÑO / COLOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SPOTS MANGA CORTA DAMA — Virgen del Valle · VELA + WEB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Virgen del Valle (Blanco)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="7" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>↳ Ref. ventas sept (curva)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="8" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="10" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL DAMA</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -723,32 +1365,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Género</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Talla</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Cantidad a producir</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>Demanda VELA</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Demanda WEB</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>Stock VELA actual</t>
         </is>
@@ -971,7 +1613,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -989,639 +1631,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>SPOTS MANGA CORTA CAB · Virgen del Valle · Blanco</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Talla</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Mix %</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Ventas sept</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Stock VELA</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Stock TALLER</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Stock WEB</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Demanda VELA</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Demanda WEB</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Demanda total</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>Stock efectivo</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>Producción sugerida</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>Cobertura VELA (días)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I3" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="K3" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="L3" s="6" t="n">
-        <v>31.5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="L4" s="6" t="n">
-        <v>12.4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>32</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>8.9</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <v>92.90000000000001</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>2XL</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="K7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>86.3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n">
-        <v>47</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="8" t="n">
-        <v>71</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="J8" s="8" t="n">
-        <v>165</v>
-      </c>
-      <c r="K8" s="9" t="n">
-        <v>35</v>
-      </c>
-      <c r="L8" s="8" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>SPOTS MANGA CORTA DAMA · Virgen del Valle · Blanco</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Talla</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Mix %</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Ventas sept</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Stock VELA</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Stock TALLER</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Stock WEB</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Demanda VELA</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Demanda WEB</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Demanda total</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>Stock efectivo</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>Producción sugerida</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>Cobertura VELA (días)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="I3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="K3" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="L3" s="6" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="L4" s="6" t="n">
-        <v>10.2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>46</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>39</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I6" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <v>13.3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n">
-        <v>64</v>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>72</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>119</v>
-      </c>
-      <c r="J7" s="8" t="n">
-        <v>102</v>
-      </c>
-      <c r="K7" s="9" t="n">
-        <v>77</v>
-      </c>
-      <c r="L7" s="8" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1631,37 +1641,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Escenario</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Días sept</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Días oct</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>WEB %</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>VELA und</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>WEB und</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>Total</t>
         </is>

</xml_diff>